<commit_message>
Fix lỗi không tính tiền khi lưu trú trong 1 ngày
</commit_message>
<xml_diff>
--- a/Documents/Master Plan(Doan3).xlsx
+++ b/Documents/Master Plan(Doan3).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Ôn tập\Năm 3\Đồ án 3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Ôn tập\Năm 3\Đồ án 3\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9CDFA36-BE84-4D7C-AE02-90ABFEC37A17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADD4A851-C9F0-4B15-A6B6-2D88D6D7DDE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -811,7 +811,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="92">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1009,7 +1009,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1338,112 +1337,112 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:71" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="83" t="s">
+      <c r="A1" s="82" t="s">
         <v>80</v>
       </c>
-      <c r="B1" s="84"/>
-      <c r="C1" s="84"/>
-      <c r="D1" s="84"/>
-      <c r="E1" s="84"/>
-      <c r="F1" s="84"/>
-      <c r="G1" s="84"/>
-      <c r="H1" s="84"/>
+      <c r="B1" s="83"/>
+      <c r="C1" s="83"/>
+      <c r="D1" s="83"/>
+      <c r="E1" s="83"/>
+      <c r="F1" s="83"/>
+      <c r="G1" s="83"/>
+      <c r="H1" s="83"/>
     </row>
     <row r="2" spans="1:71" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="85"/>
-      <c r="B2" s="85"/>
-      <c r="C2" s="85"/>
-      <c r="D2" s="85"/>
-      <c r="E2" s="85"/>
-      <c r="F2" s="85"/>
-      <c r="G2" s="85"/>
-      <c r="H2" s="85"/>
+      <c r="A2" s="84"/>
+      <c r="B2" s="84"/>
+      <c r="C2" s="84"/>
+      <c r="D2" s="84"/>
+      <c r="E2" s="84"/>
+      <c r="F2" s="84"/>
+      <c r="G2" s="84"/>
+      <c r="H2" s="84"/>
     </row>
     <row r="3" spans="1:71" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="90" t="s">
+      <c r="A3" s="89" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="90" t="s">
+      <c r="B3" s="89" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="92" t="s">
+      <c r="C3" s="91" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="92" t="s">
+      <c r="D3" s="91" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="90" t="s">
+      <c r="E3" s="89" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="90" t="s">
+      <c r="F3" s="89" t="s">
         <v>5</v>
       </c>
       <c r="G3" s="64"/>
-      <c r="H3" s="92" t="s">
+      <c r="H3" s="91" t="s">
         <v>6</v>
       </c>
-      <c r="I3" s="86" t="s">
+      <c r="I3" s="85" t="s">
         <v>7</v>
       </c>
-      <c r="J3" s="87"/>
-      <c r="K3" s="87"/>
-      <c r="L3" s="87"/>
-      <c r="M3" s="87"/>
-      <c r="N3" s="87"/>
-      <c r="O3" s="87"/>
-      <c r="P3" s="87"/>
-      <c r="Q3" s="87"/>
-      <c r="R3" s="87"/>
-      <c r="S3" s="87"/>
-      <c r="T3" s="87"/>
-      <c r="U3" s="87"/>
-      <c r="V3" s="87"/>
-      <c r="W3" s="87"/>
-      <c r="X3" s="87"/>
-      <c r="Y3" s="87"/>
-      <c r="Z3" s="87"/>
-      <c r="AA3" s="87"/>
-      <c r="AB3" s="87"/>
-      <c r="AC3" s="87"/>
-      <c r="AD3" s="87"/>
-      <c r="AE3" s="87"/>
-      <c r="AF3" s="87"/>
-      <c r="AG3" s="87"/>
-      <c r="AH3" s="87"/>
-      <c r="AI3" s="87"/>
-      <c r="AJ3" s="87"/>
-      <c r="AK3" s="87"/>
-      <c r="AL3" s="88" t="s">
+      <c r="J3" s="86"/>
+      <c r="K3" s="86"/>
+      <c r="L3" s="86"/>
+      <c r="M3" s="86"/>
+      <c r="N3" s="86"/>
+      <c r="O3" s="86"/>
+      <c r="P3" s="86"/>
+      <c r="Q3" s="86"/>
+      <c r="R3" s="86"/>
+      <c r="S3" s="86"/>
+      <c r="T3" s="86"/>
+      <c r="U3" s="86"/>
+      <c r="V3" s="86"/>
+      <c r="W3" s="86"/>
+      <c r="X3" s="86"/>
+      <c r="Y3" s="86"/>
+      <c r="Z3" s="86"/>
+      <c r="AA3" s="86"/>
+      <c r="AB3" s="86"/>
+      <c r="AC3" s="86"/>
+      <c r="AD3" s="86"/>
+      <c r="AE3" s="86"/>
+      <c r="AF3" s="86"/>
+      <c r="AG3" s="86"/>
+      <c r="AH3" s="86"/>
+      <c r="AI3" s="86"/>
+      <c r="AJ3" s="86"/>
+      <c r="AK3" s="86"/>
+      <c r="AL3" s="87" t="s">
         <v>8</v>
       </c>
-      <c r="AM3" s="89"/>
-      <c r="AN3" s="89"/>
-      <c r="AO3" s="89"/>
-      <c r="AP3" s="89"/>
-      <c r="AQ3" s="89"/>
-      <c r="AR3" s="89"/>
-      <c r="AS3" s="89"/>
-      <c r="AT3" s="89"/>
-      <c r="AU3" s="89"/>
-      <c r="AV3" s="89"/>
-      <c r="AW3" s="89"/>
-      <c r="AX3" s="89"/>
-      <c r="AY3" s="89"/>
-      <c r="AZ3" s="89"/>
-      <c r="BA3" s="89"/>
-      <c r="BB3" s="89"/>
-      <c r="BC3" s="89"/>
-      <c r="BD3" s="89"/>
-      <c r="BE3" s="89"/>
-      <c r="BF3" s="89"/>
-      <c r="BG3" s="89"/>
-      <c r="BH3" s="89"/>
-      <c r="BI3" s="89"/>
-      <c r="BJ3" s="89"/>
-      <c r="BK3" s="89"/>
-      <c r="BL3" s="89"/>
-      <c r="BM3" s="89"/>
-      <c r="BN3" s="89"/>
+      <c r="AM3" s="88"/>
+      <c r="AN3" s="88"/>
+      <c r="AO3" s="88"/>
+      <c r="AP3" s="88"/>
+      <c r="AQ3" s="88"/>
+      <c r="AR3" s="88"/>
+      <c r="AS3" s="88"/>
+      <c r="AT3" s="88"/>
+      <c r="AU3" s="88"/>
+      <c r="AV3" s="88"/>
+      <c r="AW3" s="88"/>
+      <c r="AX3" s="88"/>
+      <c r="AY3" s="88"/>
+      <c r="AZ3" s="88"/>
+      <c r="BA3" s="88"/>
+      <c r="BB3" s="88"/>
+      <c r="BC3" s="88"/>
+      <c r="BD3" s="88"/>
+      <c r="BE3" s="88"/>
+      <c r="BF3" s="88"/>
+      <c r="BG3" s="88"/>
+      <c r="BH3" s="88"/>
+      <c r="BI3" s="88"/>
+      <c r="BJ3" s="88"/>
+      <c r="BK3" s="88"/>
+      <c r="BL3" s="88"/>
+      <c r="BM3" s="88"/>
+      <c r="BN3" s="88"/>
       <c r="BO3" s="1" t="s">
         <v>9</v>
       </c>
@@ -1453,14 +1452,14 @@
       <c r="BS3" s="1"/>
     </row>
     <row r="4" spans="1:71" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="91"/>
-      <c r="B4" s="91"/>
-      <c r="C4" s="91"/>
-      <c r="D4" s="91"/>
-      <c r="E4" s="91"/>
-      <c r="F4" s="91"/>
+      <c r="A4" s="90"/>
+      <c r="B4" s="90"/>
+      <c r="C4" s="90"/>
+      <c r="D4" s="90"/>
+      <c r="E4" s="90"/>
+      <c r="F4" s="90"/>
       <c r="G4" s="65"/>
-      <c r="H4" s="91"/>
+      <c r="H4" s="90"/>
       <c r="I4" s="2">
         <v>3</v>
       </c>
@@ -1652,7 +1651,7 @@
       </c>
     </row>
     <row r="5" spans="1:71" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="80" t="s">
+      <c r="A5" s="79" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="24" t="s">
@@ -1777,7 +1776,7 @@
       <c r="D6" s="5"/>
       <c r="E6" s="11"/>
       <c r="F6" s="13" t="s">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="G6" s="8"/>
       <c r="H6" s="58"/>
@@ -1864,7 +1863,7 @@
       <c r="F7" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="G7" s="82"/>
+      <c r="G7" s="81"/>
       <c r="H7" s="59"/>
       <c r="I7" s="6"/>
       <c r="J7" s="6"/>
@@ -1949,7 +1948,7 @@
       <c r="F8" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="G8" s="82"/>
+      <c r="G8" s="81"/>
       <c r="H8" s="59"/>
       <c r="I8" s="6"/>
       <c r="J8" s="6"/>
@@ -2032,7 +2031,7 @@
         <v>46056</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="G9" s="8"/>
       <c r="H9" s="59"/>
@@ -2117,7 +2116,7 @@
         <v>46056</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="G10" s="8"/>
       <c r="H10" s="59"/>
@@ -2275,7 +2274,7 @@
       <c r="D12" s="5"/>
       <c r="E12" s="11"/>
       <c r="F12" s="13" t="s">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="G12" s="8"/>
       <c r="H12" s="59"/>
@@ -2358,9 +2357,9 @@
       </c>
       <c r="E13" s="11"/>
       <c r="F13" s="13" t="s">
-        <v>79</v>
-      </c>
-      <c r="G13" s="82"/>
+        <v>107</v>
+      </c>
+      <c r="G13" s="81"/>
       <c r="H13" s="60"/>
       <c r="I13" s="6"/>
       <c r="J13" s="6"/>
@@ -2441,9 +2440,9 @@
       </c>
       <c r="E14" s="11"/>
       <c r="F14" s="13" t="s">
-        <v>79</v>
-      </c>
-      <c r="G14" s="82"/>
+        <v>107</v>
+      </c>
+      <c r="G14" s="81"/>
       <c r="H14" s="60"/>
       <c r="I14" s="6"/>
       <c r="J14" s="6"/>
@@ -2524,9 +2523,9 @@
       </c>
       <c r="E15" s="11"/>
       <c r="F15" s="13" t="s">
-        <v>79</v>
-      </c>
-      <c r="G15" s="82"/>
+        <v>107</v>
+      </c>
+      <c r="G15" s="81"/>
       <c r="H15" s="60"/>
       <c r="I15" s="6"/>
       <c r="J15" s="6"/>
@@ -2607,7 +2606,7 @@
       </c>
       <c r="E16" s="11"/>
       <c r="F16" s="13" t="s">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="G16" s="8"/>
       <c r="H16" s="60"/>
@@ -2765,7 +2764,7 @@
       <c r="D18" s="10"/>
       <c r="E18" s="11"/>
       <c r="F18" s="13" t="s">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="G18" s="8"/>
       <c r="H18" s="60"/>
@@ -2848,7 +2847,7 @@
       </c>
       <c r="E19" s="11"/>
       <c r="F19" s="13" t="s">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="G19" s="8"/>
       <c r="H19" s="60"/>
@@ -2931,7 +2930,7 @@
       </c>
       <c r="E20" s="11"/>
       <c r="F20" s="13" t="s">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="G20" s="8"/>
       <c r="H20" s="60"/>
@@ -3014,7 +3013,7 @@
       </c>
       <c r="E21" s="11"/>
       <c r="F21" s="13" t="s">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="G21" s="8"/>
       <c r="H21" s="60"/>
@@ -3097,7 +3096,7 @@
       </c>
       <c r="E22" s="11"/>
       <c r="F22" s="13" t="s">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="G22" s="8"/>
       <c r="H22" s="60"/>
@@ -3246,16 +3245,16 @@
       <c r="A24" s="31">
         <v>4</v>
       </c>
-      <c r="B24" s="78" t="s">
+      <c r="B24" s="77" t="s">
         <v>98</v>
       </c>
-      <c r="C24" s="79" t="s">
+      <c r="C24" s="78" t="s">
         <v>69</v>
       </c>
       <c r="D24" s="70"/>
       <c r="E24" s="71"/>
       <c r="F24" s="75" t="s">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="G24" s="72"/>
       <c r="H24" s="60"/>
@@ -3335,8 +3334,8 @@
         <v>77</v>
       </c>
       <c r="E25" s="71"/>
-      <c r="F25" s="76" t="s">
-        <v>79</v>
+      <c r="F25" s="75" t="s">
+        <v>107</v>
       </c>
       <c r="G25" s="72"/>
       <c r="H25" s="60"/>
@@ -3416,8 +3415,8 @@
         <v>77</v>
       </c>
       <c r="E26" s="71"/>
-      <c r="F26" s="76" t="s">
-        <v>79</v>
+      <c r="F26" s="75" t="s">
+        <v>107</v>
       </c>
       <c r="G26" s="72"/>
       <c r="H26" s="60"/>
@@ -3497,8 +3496,8 @@
         <v>77</v>
       </c>
       <c r="E27" s="71"/>
-      <c r="F27" s="76" t="s">
-        <v>79</v>
+      <c r="F27" s="75" t="s">
+        <v>107</v>
       </c>
       <c r="G27" s="72"/>
       <c r="H27" s="60"/>
@@ -3578,8 +3577,8 @@
         <v>77</v>
       </c>
       <c r="E28" s="71"/>
-      <c r="F28" s="76" t="s">
-        <v>79</v>
+      <c r="F28" s="75" t="s">
+        <v>107</v>
       </c>
       <c r="G28" s="72"/>
       <c r="H28" s="60"/>
@@ -3665,16 +3664,16 @@
       <c r="A30" s="31">
         <v>5</v>
       </c>
-      <c r="B30" s="78" t="s">
+      <c r="B30" s="77" t="s">
         <v>90</v>
       </c>
-      <c r="C30" s="79" t="s">
+      <c r="C30" s="78" t="s">
         <v>69</v>
       </c>
       <c r="D30" s="70"/>
       <c r="E30" s="71"/>
       <c r="F30" s="76" t="s">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="G30" s="72"/>
       <c r="H30" s="60"/>
@@ -3749,13 +3748,13 @@
       <c r="B31" s="69" t="s">
         <v>99</v>
       </c>
-      <c r="C31" s="79"/>
+      <c r="C31" s="78"/>
       <c r="D31" s="70" t="s">
         <v>105</v>
       </c>
       <c r="E31" s="71"/>
       <c r="F31" s="76" t="s">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="G31" s="72"/>
       <c r="H31" s="60"/>
@@ -3836,7 +3835,7 @@
       </c>
       <c r="E32" s="71"/>
       <c r="F32" s="76" t="s">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="G32" s="72"/>
       <c r="H32" s="60"/>
@@ -3917,7 +3916,7 @@
       </c>
       <c r="E33" s="71"/>
       <c r="F33" s="76" t="s">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="G33" s="72"/>
       <c r="H33" s="60"/>
@@ -3998,7 +3997,7 @@
       </c>
       <c r="E34" s="71"/>
       <c r="F34" s="76" t="s">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="G34" s="72"/>
       <c r="H34" s="60"/>
@@ -4084,16 +4083,16 @@
       <c r="A36" s="31">
         <v>6</v>
       </c>
-      <c r="B36" s="78" t="s">
+      <c r="B36" s="77" t="s">
         <v>97</v>
       </c>
-      <c r="C36" s="79" t="s">
+      <c r="C36" s="78" t="s">
         <v>69</v>
       </c>
       <c r="D36" s="70"/>
       <c r="E36" s="71"/>
       <c r="F36" s="76" t="s">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="G36" s="72"/>
       <c r="H36" s="60"/>
@@ -4174,7 +4173,7 @@
       </c>
       <c r="E37" s="71"/>
       <c r="F37" s="76" t="s">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="G37" s="72"/>
       <c r="H37" s="60"/>
@@ -4255,7 +4254,7 @@
       </c>
       <c r="E38" s="71"/>
       <c r="F38" s="76" t="s">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="G38" s="72"/>
       <c r="H38" s="60"/>
@@ -4336,7 +4335,7 @@
       </c>
       <c r="E39" s="71"/>
       <c r="F39" s="76" t="s">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="G39" s="72"/>
       <c r="H39" s="60"/>
@@ -4417,7 +4416,7 @@
       </c>
       <c r="E40" s="71"/>
       <c r="F40" s="76" t="s">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="G40" s="72"/>
       <c r="H40" s="60"/>
@@ -4497,8 +4496,8 @@
         <v>106</v>
       </c>
       <c r="E41" s="71"/>
-      <c r="F41" s="77" t="s">
-        <v>79</v>
+      <c r="F41" s="76" t="s">
+        <v>107</v>
       </c>
       <c r="G41" s="72"/>
       <c r="H41" s="60"/>
@@ -4906,7 +4905,7 @@
         <v>55</v>
       </c>
       <c r="C47" s="53"/>
-      <c r="D47" s="81" t="s">
+      <c r="D47" s="80" t="s">
         <v>72</v>
       </c>
       <c r="E47" s="39"/>
@@ -4924,7 +4923,7 @@
         <v>56</v>
       </c>
       <c r="C48" s="53"/>
-      <c r="D48" s="81" t="s">
+      <c r="D48" s="80" t="s">
         <v>72</v>
       </c>
       <c r="E48" s="39"/>
@@ -4942,7 +4941,7 @@
         <v>57</v>
       </c>
       <c r="C49" s="53"/>
-      <c r="D49" s="81" t="s">
+      <c r="D49" s="80" t="s">
         <v>72</v>
       </c>
       <c r="E49" s="39"/>
@@ -4960,7 +4959,7 @@
         <v>58</v>
       </c>
       <c r="C50" s="53"/>
-      <c r="D50" s="81" t="s">
+      <c r="D50" s="80" t="s">
         <v>72</v>
       </c>
       <c r="E50" s="39"/>
@@ -4978,7 +4977,7 @@
         <v>59</v>
       </c>
       <c r="C51" s="53"/>
-      <c r="D51" s="81" t="s">
+      <c r="D51" s="80" t="s">
         <v>72</v>
       </c>
       <c r="E51" s="39"/>
@@ -5028,7 +5027,7 @@
         <v>62</v>
       </c>
       <c r="C54" s="53"/>
-      <c r="D54" s="81" t="s">
+      <c r="D54" s="80" t="s">
         <v>72</v>
       </c>
       <c r="E54" s="39"/>
@@ -5046,7 +5045,7 @@
         <v>63</v>
       </c>
       <c r="C55" s="53"/>
-      <c r="D55" s="81" t="s">
+      <c r="D55" s="80" t="s">
         <v>72</v>
       </c>
       <c r="E55" s="39"/>
@@ -5064,7 +5063,7 @@
         <v>64</v>
       </c>
       <c r="C56" s="53"/>
-      <c r="D56" s="81" t="s">
+      <c r="D56" s="80" t="s">
         <v>72</v>
       </c>
       <c r="E56" s="39"/>
@@ -5082,7 +5081,7 @@
         <v>65</v>
       </c>
       <c r="C57" s="53"/>
-      <c r="D57" s="81" t="s">
+      <c r="D57" s="80" t="s">
         <v>72</v>
       </c>
       <c r="E57" s="39"/>
@@ -5100,7 +5099,7 @@
         <v>66</v>
       </c>
       <c r="C58" s="53"/>
-      <c r="D58" s="81" t="s">
+      <c r="D58" s="80" t="s">
         <v>72</v>
       </c>
       <c r="E58" s="39"/>
@@ -5118,7 +5117,7 @@
         <v>67</v>
       </c>
       <c r="C59" s="53"/>
-      <c r="D59" s="81" t="s">
+      <c r="D59" s="80" t="s">
         <v>72</v>
       </c>
       <c r="E59" s="39"/>
@@ -5136,7 +5135,7 @@
         <v>68</v>
       </c>
       <c r="C60" s="53"/>
-      <c r="D60" s="81" t="s">
+      <c r="D60" s="80" t="s">
         <v>72</v>
       </c>
       <c r="E60" s="39"/>
@@ -6038,7 +6037,7 @@
     <mergeCell ref="H3:H4"/>
   </mergeCells>
   <phoneticPr fontId="11" type="noConversion"/>
-  <conditionalFormatting sqref="F6:F10 F11:G11 F12:F16 F17:G17 F18:F22 F23:G23 F24:F28 F29:G29 F30:F34 F35:G35 F36:F41 F42:G45 F46:F51 F52:G52">
+  <conditionalFormatting sqref="F11:G11 F17:G17 F23:G23 F29:G29 F35:G35 F42:G45 F46:F51 F52:G52 F6:F10 F12:F16 F18:F22 F24:F28 F30:F34 F36:F41">
     <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="Đã hoàn thành">
       <formula>NOT(ISERROR(SEARCH(("Đã hoàn thành"),(F6))))</formula>
     </cfRule>
@@ -6069,7 +6068,7 @@
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H44:H45 H6:H28 H30:H34 H36:H42" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"10%,20%,30%,40%,50%,60%,70%,80%,90%,100%"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="G52 G11 G17 G42:G45 G23 G29 F6:F60 G35" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="G52 G11 G17 G42:G45 G23 G29 G35 F6:F60" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Đang thực hiện,Đã hoàn thành"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>